<commit_message>
Fix: remove 'Turkish' word from EN description, regenerate KML
</commit_message>
<xml_diff>
--- a/الأماكن مع الترجمة.xlsx
+++ b/الأماكن مع الترجمة.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abn-a\Desktop\nabawi_maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9DCAD0-2970-413B-A270-002309FD1289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0C086F-8C24-42E0-8840-104071E70759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -304,9 +304,6 @@
     <t>مسجد القبلتين من المساجد التاريخية البارزة في المدينة المنورة، ويقع في منطقة بني سلمة شمال غربي المسجد النبوي بالقرب من وادي العقيق. يعود اسمه إلى الحدث العظيم الذي ارتبط به، وهو تحويل القبلة من بيت المقدس إلى الكعبة المشرفة أثناء صلاة المسلمين فيه، فاشتهر منذ ذلك الحين بمسجد القبلتين. ويُعد من المساجد التي صلى فيها النبي ﷺ، وقد شهد عبر تاريخه عدة مراحل من الترميم والتجديد، بدءًا من بنائه البسيط في العصور الأولى وصولًا إلى إعادة بنائه وتوسعته في عهد المملكة العربية السعودية ، ليصبح مسجدًا متكامل المرافق يتسع لأعداد كبيرة من المصلين.</t>
   </si>
   <si>
-    <t>Masjid Al-Qiblatayn (The Mosque of the Two Qiblas) is one of the prominent historical mosques in Al-Madinah Al-Munawwarah, located in the Bani Salama area, northwest of the Prophet's Mosque, near Wadi Al-Aqeeq. Its name goes back to the great event associated with it, which is the changing of the Qibla (direction of prayer) from Bait Al-Maqdis (Jerusalem) to the Honorable Kaaba while Muslims were praying in it, so it became famous since then as the Mosque of the Two Qiblas. It is considered one of the mosques in which the Prophet ﷺ prayed, and it has witnessed throughout its history several stages of restoration and renovation, starting from its simple construction in the early eras, all the way to its reconstruction and expansion during the era of the Kingdom of Saudi Arabia, to become a mosque with integrated facilities that accommodates large numbers of worshipers. Turkish</t>
-  </si>
-  <si>
     <t>Mescid-i Kıbleteyn (İki Kıbleli Mescit), Medine-i Münevvere'deki önde gelen tarihi mescitlerden biridir ve Mescid-i Nebevi'nin kuzeybatısında, Akik Vadisi yakınlarındaki Beni Seleme bölgesinde yer almaktadır. Adı, onunla ilişkilendirilen büyük bir olaya, yani Müslümanların içinde namaz kıldıkları sırada kıblenin Beytü'l-Makdis'ten (Kudüs) Kâbe-i Müşerrefe'ye çevrilmesine dayanır ve o zamandan beri Mescid-i Kıbleteyn olarak meşhur olmuştur. Hz. Peygamber'in ﷺ içinde namaz kıldığı mescitlerden biri olarak kabul edilir ve tarihi boyunca, ilk çağlardaki basit yapısından başlayarak Suudi Arabistan Krallığı döneminde yeniden inşa edilip genişletilmesine kadar birçok restorasyon ve yenileme aşamasına tanık olmuş, böylece çok sayıda ibadet edeni barındıran tam donanımlı tesisleri olan bir mescit haline gelmiştir.</t>
   </si>
   <si>
@@ -1235,6 +1232,9 @@
   </si>
   <si>
     <t>Salah satu tempat di mana Nabi ﷺ shalat dan berpesan tentang ahli baitnya (keluarganya), beliau shalallahu 'alaihi wa sallam bersabda: "Ketahuilah wahai manusia, sesungguhnya aku hanyalah seorang manusia, hampir tiba saatnya utusan Tuhanku (malaikat maut) datang lalu aku memenuhinya. Dan aku meninggalkan di tengah-tengah kalian dua hal yang berat: yang pertama adalah Kitabullah, di dalamnya terdapat petunjuk dan cahaya, maka pegang teguhlah Kitabullah dan berpeganglah padanya." Beliau mendorong untuk berpegang pada Kitabullah dan menganjurkannya, kemudian beliau bersabda: "Dan ahli baitku; aku ingatkan kalian kepada Allah tentang ahli baitku, aku ingatkan kalian kepada Allah tentang ahli baitku, aku ingatkan kalian kepada Allah tentang ahli baitku."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masjid Al-Qiblatayn (The Mosque of the Two Qiblas) is one of the prominent historical mosques in Al-Madinah Al-Munawwarah, located in the Bani Salama area, northwest of the Prophet's Mosque, near Wadi Al-Aqeeq. Its name goes back to the great event associated with it, which is the changing of the Qibla (direction of prayer) from Bait Al-Maqdis (Jerusalem) to the Honorable Kaaba while Muslims were praying in it, so it became famous since then as the Mosque of the Two Qiblas. It is considered one of the mosques in which the Prophet ﷺ prayed, and it has witnessed throughout its history several stages of restoration and renovation, starting from its simple construction in the early eras, all the way to its reconstruction and expansion during the era of the Kingdom of Saudi Arabia, to become a mosque with integrated facilities that accommodates large numbers of worshipers. </t>
   </si>
 </sst>
 </file>
@@ -1635,13 +1635,13 @@
         <v>93</v>
       </c>
       <c r="C2" t="s">
+        <v>404</v>
+      </c>
+      <c r="D2" t="s">
         <v>94</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>95</v>
-      </c>
-      <c r="E2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1649,16 +1649,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" t="s">
         <v>97</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>98</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>99</v>
-      </c>
-      <c r="E3" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1666,16 +1666,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" t="s">
         <v>101</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>102</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>103</v>
-      </c>
-      <c r="E4" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1683,16 +1683,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" t="s">
         <v>105</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>106</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>107</v>
-      </c>
-      <c r="E5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1700,16 +1700,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" t="s">
         <v>109</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>110</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>111</v>
-      </c>
-      <c r="E6" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -1717,16 +1717,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
         <v>113</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>114</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>115</v>
-      </c>
-      <c r="E7" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -1734,16 +1734,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" t="s">
         <v>117</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>118</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>119</v>
-      </c>
-      <c r="E8" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1754,13 +1754,13 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" t="s">
         <v>121</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>122</v>
-      </c>
-      <c r="E9" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -1768,16 +1768,16 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" t="s">
         <v>124</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>125</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>126</v>
-      </c>
-      <c r="E10" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1785,16 +1785,16 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" t="s">
         <v>128</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>129</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>130</v>
-      </c>
-      <c r="E11" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -1805,10 +1805,10 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D12" t="s">
         <v>132</v>
-      </c>
-      <c r="D12" t="s">
-        <v>133</v>
       </c>
       <c r="E12" t="s">
         <v>18</v>
@@ -1819,16 +1819,16 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
+        <v>133</v>
+      </c>
+      <c r="C13" t="s">
         <v>134</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>135</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>136</v>
-      </c>
-      <c r="E13" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -1839,13 +1839,13 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" t="s">
         <v>138</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>139</v>
-      </c>
-      <c r="E14" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1856,13 +1856,13 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
+        <v>140</v>
+      </c>
+      <c r="D15" t="s">
         <v>141</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>142</v>
-      </c>
-      <c r="E15" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -1873,13 +1873,13 @@
         <v>25</v>
       </c>
       <c r="C16" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" t="s">
         <v>144</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>145</v>
-      </c>
-      <c r="E16" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1890,13 +1890,13 @@
         <v>27</v>
       </c>
       <c r="C17" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" t="s">
         <v>147</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>148</v>
-      </c>
-      <c r="E17" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -1907,13 +1907,13 @@
         <v>29</v>
       </c>
       <c r="C18" t="s">
+        <v>149</v>
+      </c>
+      <c r="D18" t="s">
         <v>150</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>151</v>
-      </c>
-      <c r="E18" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1924,13 +1924,13 @@
         <v>31</v>
       </c>
       <c r="C19" t="s">
+        <v>152</v>
+      </c>
+      <c r="D19" t="s">
         <v>153</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>154</v>
-      </c>
-      <c r="E19" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1938,16 +1938,16 @@
         <v>32</v>
       </c>
       <c r="B20" t="s">
+        <v>155</v>
+      </c>
+      <c r="C20" t="s">
         <v>156</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>157</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>158</v>
-      </c>
-      <c r="E20" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -1958,13 +1958,13 @@
         <v>34</v>
       </c>
       <c r="C21" t="s">
+        <v>159</v>
+      </c>
+      <c r="D21" t="s">
         <v>160</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>161</v>
-      </c>
-      <c r="E21" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1975,13 +1975,13 @@
         <v>36</v>
       </c>
       <c r="C22" t="s">
+        <v>162</v>
+      </c>
+      <c r="D22" t="s">
         <v>163</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>164</v>
-      </c>
-      <c r="E22" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1989,16 +1989,16 @@
         <v>37</v>
       </c>
       <c r="B23" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" t="s">
         <v>166</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>167</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>168</v>
-      </c>
-      <c r="E23" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -2009,13 +2009,13 @@
         <v>39</v>
       </c>
       <c r="C24" t="s">
+        <v>169</v>
+      </c>
+      <c r="D24" t="s">
         <v>170</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>171</v>
-      </c>
-      <c r="E24" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -2023,16 +2023,16 @@
         <v>40</v>
       </c>
       <c r="B25" t="s">
+        <v>172</v>
+      </c>
+      <c r="C25" t="s">
         <v>173</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>174</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>175</v>
-      </c>
-      <c r="E25" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -2040,16 +2040,16 @@
         <v>41</v>
       </c>
       <c r="B26" t="s">
+        <v>176</v>
+      </c>
+      <c r="C26" t="s">
         <v>177</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>178</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>179</v>
-      </c>
-      <c r="E26" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -2060,13 +2060,13 @@
         <v>43</v>
       </c>
       <c r="C27" t="s">
+        <v>180</v>
+      </c>
+      <c r="D27" t="s">
         <v>181</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>182</v>
-      </c>
-      <c r="E27" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -2074,16 +2074,16 @@
         <v>44</v>
       </c>
       <c r="B28" t="s">
+        <v>183</v>
+      </c>
+      <c r="C28" t="s">
         <v>184</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>185</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>186</v>
-      </c>
-      <c r="E28" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -2091,16 +2091,16 @@
         <v>45</v>
       </c>
       <c r="B29" t="s">
+        <v>187</v>
+      </c>
+      <c r="C29" t="s">
         <v>188</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>189</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>190</v>
-      </c>
-      <c r="E29" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -2111,13 +2111,13 @@
         <v>47</v>
       </c>
       <c r="C30" t="s">
+        <v>191</v>
+      </c>
+      <c r="D30" t="s">
         <v>192</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>193</v>
-      </c>
-      <c r="E30" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -2125,16 +2125,16 @@
         <v>48</v>
       </c>
       <c r="B31" t="s">
+        <v>194</v>
+      </c>
+      <c r="C31" t="s">
         <v>195</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>196</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>197</v>
-      </c>
-      <c r="E31" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -2145,13 +2145,13 @@
         <v>50</v>
       </c>
       <c r="C32" t="s">
+        <v>198</v>
+      </c>
+      <c r="D32" t="s">
         <v>199</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>200</v>
-      </c>
-      <c r="E32" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -2162,13 +2162,13 @@
         <v>52</v>
       </c>
       <c r="C33" t="s">
+        <v>201</v>
+      </c>
+      <c r="D33" t="s">
         <v>202</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>203</v>
-      </c>
-      <c r="E33" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -2176,33 +2176,33 @@
         <v>53</v>
       </c>
       <c r="B34" t="s">
+        <v>204</v>
+      </c>
+      <c r="C34" t="s">
         <v>205</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>206</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>207</v>
-      </c>
-      <c r="E34" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>208</v>
+      </c>
+      <c r="B35" t="s">
         <v>209</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>210</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>211</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>212</v>
-      </c>
-      <c r="E35" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -2210,16 +2210,16 @@
         <v>54</v>
       </c>
       <c r="B36" t="s">
+        <v>213</v>
+      </c>
+      <c r="C36" t="s">
         <v>214</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>215</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>216</v>
-      </c>
-      <c r="E36" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -2227,16 +2227,16 @@
         <v>55</v>
       </c>
       <c r="B37" t="s">
+        <v>221</v>
+      </c>
+      <c r="C37" t="s">
         <v>222</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>223</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>224</v>
-      </c>
-      <c r="E37" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -2244,16 +2244,16 @@
         <v>56</v>
       </c>
       <c r="B38" t="s">
+        <v>217</v>
+      </c>
+      <c r="C38" t="s">
         <v>218</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>219</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>220</v>
-      </c>
-      <c r="E38" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -2264,13 +2264,13 @@
         <v>58</v>
       </c>
       <c r="C39" t="s">
+        <v>225</v>
+      </c>
+      <c r="D39" t="s">
         <v>226</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>227</v>
-      </c>
-      <c r="E39" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -2298,13 +2298,13 @@
         <v>65</v>
       </c>
       <c r="C41" t="s">
+        <v>228</v>
+      </c>
+      <c r="D41" t="s">
         <v>229</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>230</v>
-      </c>
-      <c r="E41" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -2315,13 +2315,13 @@
         <v>67</v>
       </c>
       <c r="C42" t="s">
+        <v>231</v>
+      </c>
+      <c r="D42" t="s">
         <v>232</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>233</v>
-      </c>
-      <c r="E42" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -2332,13 +2332,13 @@
         <v>69</v>
       </c>
       <c r="C43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D43" t="s">
         <v>235</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>236</v>
-      </c>
-      <c r="E43" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -2349,13 +2349,13 @@
         <v>71</v>
       </c>
       <c r="C44" t="s">
+        <v>237</v>
+      </c>
+      <c r="D44" t="s">
         <v>238</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>239</v>
-      </c>
-      <c r="E44" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -2363,16 +2363,16 @@
         <v>72</v>
       </c>
       <c r="B45" t="s">
+        <v>240</v>
+      </c>
+      <c r="C45" t="s">
         <v>241</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>242</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>243</v>
-      </c>
-      <c r="E45" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -2383,13 +2383,13 @@
         <v>74</v>
       </c>
       <c r="C46" t="s">
+        <v>244</v>
+      </c>
+      <c r="D46" t="s">
         <v>245</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>246</v>
-      </c>
-      <c r="E46" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
@@ -2400,13 +2400,13 @@
         <v>76</v>
       </c>
       <c r="C47" t="s">
+        <v>247</v>
+      </c>
+      <c r="D47" t="s">
         <v>248</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>249</v>
-      </c>
-      <c r="E47" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -2414,16 +2414,16 @@
         <v>77</v>
       </c>
       <c r="B48" t="s">
+        <v>250</v>
+      </c>
+      <c r="C48" t="s">
         <v>251</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>252</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>253</v>
-      </c>
-      <c r="E48" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -2431,16 +2431,16 @@
         <v>78</v>
       </c>
       <c r="B49" t="s">
+        <v>254</v>
+      </c>
+      <c r="C49" t="s">
         <v>255</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>256</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>257</v>
-      </c>
-      <c r="E49" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -2448,16 +2448,16 @@
         <v>79</v>
       </c>
       <c r="B50" t="s">
+        <v>258</v>
+      </c>
+      <c r="C50" t="s">
         <v>259</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>260</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>261</v>
-      </c>
-      <c r="E50" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
@@ -2465,16 +2465,16 @@
         <v>80</v>
       </c>
       <c r="B51" t="s">
+        <v>263</v>
+      </c>
+      <c r="C51" t="s">
+        <v>262</v>
+      </c>
+      <c r="D51" t="s">
         <v>264</v>
       </c>
-      <c r="C51" t="s">
-        <v>263</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>265</v>
-      </c>
-      <c r="E51" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
@@ -2482,16 +2482,16 @@
         <v>81</v>
       </c>
       <c r="B52" t="s">
+        <v>266</v>
+      </c>
+      <c r="C52" t="s">
         <v>267</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>268</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>269</v>
-      </c>
-      <c r="E52" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
@@ -2499,16 +2499,16 @@
         <v>82</v>
       </c>
       <c r="B53" t="s">
+        <v>270</v>
+      </c>
+      <c r="C53" t="s">
         <v>271</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>272</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>273</v>
-      </c>
-      <c r="E53" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
@@ -2516,16 +2516,16 @@
         <v>83</v>
       </c>
       <c r="B54" t="s">
+        <v>274</v>
+      </c>
+      <c r="C54" t="s">
         <v>275</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>276</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>277</v>
-      </c>
-      <c r="E54" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
@@ -2533,16 +2533,16 @@
         <v>84</v>
       </c>
       <c r="B55" t="s">
+        <v>278</v>
+      </c>
+      <c r="C55" t="s">
         <v>279</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>280</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>281</v>
-      </c>
-      <c r="E55" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
@@ -2553,13 +2553,13 @@
         <v>86</v>
       </c>
       <c r="C56" t="s">
+        <v>282</v>
+      </c>
+      <c r="D56" t="s">
         <v>283</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>284</v>
-      </c>
-      <c r="E56" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
@@ -2570,13 +2570,13 @@
         <v>88</v>
       </c>
       <c r="C57" t="s">
+        <v>285</v>
+      </c>
+      <c r="D57" t="s">
         <v>286</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>287</v>
-      </c>
-      <c r="E57" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
@@ -2587,13 +2587,13 @@
         <v>90</v>
       </c>
       <c r="C58" t="s">
+        <v>288</v>
+      </c>
+      <c r="D58" t="s">
         <v>289</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>290</v>
-      </c>
-      <c r="E58" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
@@ -2604,387 +2604,387 @@
         <v>92</v>
       </c>
       <c r="C59" t="s">
+        <v>291</v>
+      </c>
+      <c r="D59" t="s">
         <v>292</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>293</v>
-      </c>
-      <c r="E59" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>294</v>
+      </c>
+      <c r="B60" t="s">
         <v>295</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>296</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>297</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>298</v>
-      </c>
-      <c r="E60" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>299</v>
+      </c>
+      <c r="B61" t="s">
         <v>300</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>301</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
         <v>302</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>303</v>
-      </c>
-      <c r="E61" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>304</v>
+      </c>
+      <c r="B62" t="s">
         <v>305</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>306</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>307</v>
       </c>
-      <c r="D62" t="s">
+      <c r="E62" t="s">
         <v>308</v>
-      </c>
-      <c r="E62" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
+        <v>309</v>
+      </c>
+      <c r="B63" t="s">
         <v>310</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
         <v>311</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>312</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>313</v>
-      </c>
-      <c r="E63" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
+        <v>314</v>
+      </c>
+      <c r="B64" t="s">
         <v>315</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>316</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
         <v>317</v>
       </c>
-      <c r="D64" t="s">
+      <c r="E64" t="s">
         <v>318</v>
-      </c>
-      <c r="E64" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
+        <v>320</v>
+      </c>
+      <c r="B65" t="s">
+        <v>319</v>
+      </c>
+      <c r="C65" t="s">
         <v>321</v>
       </c>
-      <c r="B65" t="s">
-        <v>320</v>
-      </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>322</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>323</v>
-      </c>
-      <c r="E65" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
+        <v>324</v>
+      </c>
+      <c r="B66" t="s">
         <v>325</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>326</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>327</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>328</v>
-      </c>
-      <c r="E66" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>329</v>
+      </c>
+      <c r="B67" t="s">
         <v>330</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>331</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>332</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>333</v>
-      </c>
-      <c r="E67" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>334</v>
+      </c>
+      <c r="B68" t="s">
         <v>335</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>336</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>337</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>338</v>
-      </c>
-      <c r="E68" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
+        <v>339</v>
+      </c>
+      <c r="B69" t="s">
         <v>340</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>341</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>342</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
         <v>343</v>
-      </c>
-      <c r="E69" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
+        <v>345</v>
+      </c>
+      <c r="B70" t="s">
+        <v>344</v>
+      </c>
+      <c r="C70" t="s">
         <v>346</v>
       </c>
-      <c r="B70" t="s">
-        <v>345</v>
-      </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>347</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
         <v>348</v>
-      </c>
-      <c r="E70" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
+        <v>349</v>
+      </c>
+      <c r="B71" t="s">
         <v>350</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>351</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>352</v>
       </c>
-      <c r="D71" t="s">
+      <c r="E71" t="s">
         <v>353</v>
-      </c>
-      <c r="E71" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
+        <v>354</v>
+      </c>
+      <c r="B72" t="s">
         <v>355</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>356</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>357</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
         <v>358</v>
-      </c>
-      <c r="E72" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
+        <v>359</v>
+      </c>
+      <c r="B73" t="s">
         <v>360</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>361</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>362</v>
       </c>
-      <c r="D73" t="s">
+      <c r="E73" t="s">
         <v>363</v>
-      </c>
-      <c r="E73" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
+        <v>364</v>
+      </c>
+      <c r="B74" t="s">
         <v>365</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>366</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>367</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>368</v>
-      </c>
-      <c r="E74" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
+        <v>369</v>
+      </c>
+      <c r="B75" t="s">
         <v>370</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>371</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>372</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>373</v>
-      </c>
-      <c r="E75" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
+        <v>374</v>
+      </c>
+      <c r="B76" t="s">
+        <v>376</v>
+      </c>
+      <c r="C76" t="s">
         <v>375</v>
       </c>
-      <c r="B76" t="s">
+      <c r="D76" t="s">
         <v>377</v>
       </c>
-      <c r="C76" t="s">
-        <v>376</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>378</v>
-      </c>
-      <c r="E76" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
+        <v>379</v>
+      </c>
+      <c r="B77" t="s">
         <v>380</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>381</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>382</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
         <v>383</v>
-      </c>
-      <c r="E77" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
+        <v>384</v>
+      </c>
+      <c r="B78" t="s">
         <v>385</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>386</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>387</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
         <v>388</v>
-      </c>
-      <c r="E78" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
+        <v>389</v>
+      </c>
+      <c r="B79" t="s">
         <v>390</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C79" t="s">
         <v>391</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>392</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
         <v>393</v>
-      </c>
-      <c r="E79" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
+        <v>394</v>
+      </c>
+      <c r="B80" t="s">
         <v>395</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>396</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>397</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>398</v>
-      </c>
-      <c r="E80" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
+        <v>399</v>
+      </c>
+      <c r="B81" t="s">
         <v>400</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>401</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>402</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>403</v>
-      </c>
-      <c r="E81" t="s">
-        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>